<commit_message>
Update clients data file and deploy
</commit_message>
<xml_diff>
--- a/public/clients.xlsx
+++ b/public/clients.xlsx
@@ -1,42 +1,107 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\For Other\fehed\Tech\TechInnoSphere-Single\TechInnoSphere\public\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6794F242-B3A6-4CE9-9FCB-01CF94514054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+  <si>
+    <t>Client Name</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Latitude</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>Project Count</t>
+  </si>
+  <si>
+    <t>News AI</t>
+  </si>
+  <si>
+    <t>Austria</t>
+  </si>
+  <si>
+    <t>Vienna</t>
+  </si>
+  <si>
+    <t>Ace Consultants</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>Toronto</t>
+  </si>
+  <si>
+    <t>Shahji Shipping</t>
+  </si>
+  <si>
+    <t>UAE</t>
+  </si>
+  <si>
+    <t>Dubai</t>
+  </si>
+  <si>
+    <t>Kira Ledgers</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Chanakya School</t>
+  </si>
+  <si>
+    <t>Palghar</t>
+  </si>
+  <si>
+    <t>PMK Steel</t>
+  </si>
+  <si>
+    <t>Punjab</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -64,14 +129,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,152 +475,158 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.8984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.296875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Client Name</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Country</v>
-      </c>
-      <c r="C1" t="str">
-        <v>City</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Latitude</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Longitude</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Project Count</v>
+    <row r="1" spans="1:6" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>News AI</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Austria</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Vienna</v>
-      </c>
-      <c r="D2">
-        <v>48.2082</v>
-      </c>
-      <c r="E2">
-        <v>16.3738</v>
-      </c>
-      <c r="F2">
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="2">
+        <v>28.613900000000001</v>
+      </c>
+      <c r="E2" s="2">
+        <v>77.209000000000003</v>
+      </c>
+      <c r="F2" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Ace Consultants</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Canada</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Toronto</v>
-      </c>
-      <c r="D3">
-        <v>43.65107</v>
-      </c>
-      <c r="E3">
-        <v>-79.347015</v>
-      </c>
-      <c r="F3">
+    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2">
+        <v>43.651069999999997</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-79.347014999999999</v>
+      </c>
+      <c r="F3" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Shahji Shipping</v>
-      </c>
-      <c r="B4" t="str">
-        <v>UAE</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Dubai</v>
-      </c>
-      <c r="D4">
-        <v>25.2048</v>
-      </c>
-      <c r="E4">
-        <v>55.2708</v>
-      </c>
-      <c r="F4">
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2">
+        <v>25.204799999999999</v>
+      </c>
+      <c r="E4" s="2">
+        <v>55.270800000000001</v>
+      </c>
+      <c r="F4" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Kira Ledgers</v>
-      </c>
-      <c r="B5" t="str">
-        <v>India</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Mumbai</v>
-      </c>
-      <c r="D5">
-        <v>19.076</v>
-      </c>
-      <c r="E5">
-        <v>72.8777</v>
-      </c>
-      <c r="F5">
+    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2">
+        <v>48.208199999999998</v>
+      </c>
+      <c r="E5" s="2">
+        <v>16.373799999999999</v>
+      </c>
+      <c r="F5" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Chanakya School</v>
-      </c>
-      <c r="B6" t="str">
-        <v>India</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Palghar</v>
-      </c>
-      <c r="D6">
+    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2">
         <v>19.6967</v>
       </c>
-      <c r="E6">
-        <v>72.7699</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="2">
+        <v>72.769900000000007</v>
+      </c>
+      <c r="F6" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>PMK Steel</v>
-      </c>
-      <c r="B7" t="str">
-        <v>India</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Punjab</v>
-      </c>
-      <c r="D7">
-        <v>31.1471</v>
-      </c>
-      <c r="E7">
-        <v>75.3412</v>
-      </c>
-      <c r="F7">
+    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2">
+        <v>31.147099999999998</v>
+      </c>
+      <c r="E7" s="2">
+        <v>75.341200000000001</v>
+      </c>
+      <c r="F7" s="2">
         <v>1</v>
       </c>
     </row>
+    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>